<commit_message>
Adjusted the legends of the plots
</commit_message>
<xml_diff>
--- a/results/no_unpooling/plots/06_gap_table.xlsx
+++ b/results/no_unpooling/plots/06_gap_table.xlsx
@@ -445,22 +445,22 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>SAGC (Greedy)</t>
+          <t>Song+SAGC (Greedy)</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>SAGC (Sampling)</t>
+          <t>Song+SAGC (Sampling)</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>NoPooling (Greedy)</t>
+          <t>Song (Greedy)</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>NoPooling (Sampling)</t>
+          <t>Song (Sampling)</t>
         </is>
       </c>
     </row>

</xml_diff>